<commit_message>
GLOB-1144: Enabled the policy delinquency information view, available in both summarized and detailed formats.
</commit_message>
<xml_diff>
--- a/Documentación/brecha vida Colectivo.xlsx
+++ b/Documentación/brecha vida Colectivo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398AF97D-4F3E-414A-97CC-5444EE7AAB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{629FA759-8D67-4693-921D-F28765FC8007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Vida - Emision" sheetId="3" r:id="rId1"/>
@@ -40,14 +40,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="109">
   <si>
     <t>Coaseguro</t>
   </si>
   <si>
-    <t>Documentos</t>
-  </si>
-  <si>
     <t>Módulo / Sección</t>
   </si>
   <si>
@@ -93,18 +90,9 @@
     <t>⚠️</t>
   </si>
   <si>
-    <t>Datos generales de la fianza</t>
-  </si>
-  <si>
-    <t>Objeto asegurado Fianza</t>
-  </si>
-  <si>
     <t>Si</t>
   </si>
   <si>
-    <t>Cotización</t>
-  </si>
-  <si>
     <t>Reaseguro</t>
   </si>
   <si>
@@ -115,9 +103,6 @@
   </si>
   <si>
     <t>Configurar</t>
-  </si>
-  <si>
-    <t>Facturación</t>
   </si>
   <si>
     <t>Formato endoso</t>
@@ -168,9 +153,6 @@
     <t>Actualmente no configurado en SIS9, pero expresan que se requiere porque es importante para el ramo
 Ver si al crear la recuperacón en reclamo el sistema cotnabiliza
 Recuperación se crea en reclamos y luego aparece en caja y se permite cobrar usando su respectiva transacción</t>
-  </si>
-  <si>
-    <t>1. Se registra suma comercial y de reaseguro para configurar reaseguro</t>
   </si>
   <si>
     <t>1. Coberturas no tienen tarifas automáticas, todo se registra manualmente en la cobertura, tanto prima como suma
@@ -195,9 +177,6 @@
 2. Se afecta únicamente el CP y no el excedente
 3. Distribuyen recargo/descuento entre todas las coberturas
 4. Validar reaseguro en el endoso</t>
-  </si>
-  <si>
-    <t>Prima de provisión</t>
   </si>
   <si>
     <t xml:space="preserve">1. Mismo % de impuesto 5%
@@ -273,28 +252,11 @@
     <t>Pendiente de explicación por parte de Luis</t>
   </si>
   <si>
-    <t>Datos generales del ramo (Validar información)
-Vigencia debe ser un mes y no afectar la prorrata
-Colectivo de empleados no está en uso (referencia)</t>
-  </si>
-  <si>
     <t>Sis9 tiene una carga masiva de reclamos según un formato
 Jessica envió formato para la carga, se debe revisar el proceso y lo que hace</t>
   </si>
   <si>
-    <t>Tiene validación de tomador fijo</t>
-  </si>
-  <si>
     <t>GAP Progreso</t>
-  </si>
-  <si>
-    <t>Validar edad de ingreso</t>
-  </si>
-  <si>
-    <t>Prima no Cambia</t>
-  </si>
-  <si>
-    <t>Facturación - GAP Progreso</t>
   </si>
   <si>
     <t>Se emite por certificados, se debe crear la grupal
@@ -304,9 +266,6 @@
 Aportes se restan el valor original para calcular el valor faltante</t>
   </si>
   <si>
-    <t>OA - GAP Progreso</t>
-  </si>
-  <si>
     <t xml:space="preserve"> GAP Progreso</t>
   </si>
   <si>
@@ -333,10 +292,6 @@
   </si>
   <si>
     <t>No está activo, no se validarían endosos, solo cancelación</t>
-  </si>
-  <si>
-    <t>SE emite como colectivo, se pone la cantidad de personas que son las que van a facturarse
-Jessica evaluará el producto, solo se migrará el dato y no se configurará en sis11 (aunque ya lo hicimos)</t>
   </si>
   <si>
     <t>Jessica comenta que es importante para ellos ver un estado de vencida de pólizas</t>
@@ -353,9 +308,6 @@
     <t>Configurar y Desarrollar</t>
   </si>
   <si>
-    <t>Datos de la póliza</t>
-  </si>
-  <si>
     <t>Revisar y evaluar</t>
   </si>
   <si>
@@ -405,6 +357,56 @@
   </si>
   <si>
     <t>Pagos</t>
+  </si>
+  <si>
+    <t>Registro de datos generales de la póliza</t>
+  </si>
+  <si>
+    <t>Validación del registro del objeto asegurado de la póliza</t>
+  </si>
+  <si>
+    <t>Criterios de validación</t>
+  </si>
+  <si>
+    <t>1. Validar datos generales de la emisión de cada producto según especificaciones esperadas.
+2. La vigencia de la póliza debe ser un mes y no aplica prorrata a los cálculos de la prima emitida
+3. Colectivo de empleados no está en uso (referencia)</t>
+  </si>
+  <si>
+    <t>En productos de VC se registra suma comercial y de reaseguro para configurar reaseguro</t>
+  </si>
+  <si>
+    <t>Cotización de la póliza (primas)</t>
+  </si>
+  <si>
+    <t>Generación de documentos de la póliza, oferta, póliza, etc</t>
+  </si>
+  <si>
+    <t>Visualización y validación de facturación de la póliza</t>
+  </si>
+  <si>
+    <t>Generación de pólizas en concepto de Prima de provisión</t>
+  </si>
+  <si>
+    <t>Registro y validación del objeto asegurado en producto GAP Progreso</t>
+  </si>
+  <si>
+    <t>Prima no Cambia en cada renovación
+Validar edades de ingreso y suscripción
+Existe una validación en sis9 sobre el tomador fijo del producto</t>
+  </si>
+  <si>
+    <t>Condiciones - GAP Progreso</t>
+  </si>
+  <si>
+    <t>Emisión producto CV 2016-1</t>
+  </si>
+  <si>
+    <t>SE emite como colectivo, se pone la cantidad de personas que son las que van a facturarse
+Jessica evaluará el producto, solo se migrará el dato, el producto se configurará para efectos de migración pero no habrá criterios de aceptación sobre el mismo por que ya no se emite</t>
+  </si>
+  <si>
+    <t>Datos de la póliza (Estado vencido)</t>
   </si>
 </sst>
 </file>
@@ -448,7 +450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -486,7 +488,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -804,11 +805,11 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.28515625" style="4" bestFit="1" customWidth="1"/>
@@ -819,340 +820,288 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>8</v>
-      </c>
       <c r="H1" s="5" t="s">
-        <v>9</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>94</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>95</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>24</v>
-      </c>
       <c r="H4" s="6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>100</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="F5" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>101</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>48</v>
+        <v>13</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>90</v>
-      </c>
       <c r="H8" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>74</v>
+        <v>13</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>105</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>71</v>
+        <v>13</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>106</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>72</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>71</v>
+        <v>13</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>108</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1178,158 +1127,158 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1354,184 +1303,184 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>8</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>99</v>
-      </c>
       <c r="H7" s="1" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1561,403 +1510,403 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="7" t="s">
         <v>8</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>12</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
       <c r="H5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>35</v>
-      </c>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="H6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E10" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H10" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E12" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H12" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="E13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H16" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1980,163 +1929,163 @@
     <col min="5" max="5" width="6.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="82.7109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="82.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>